<commit_message>
obbba and tariff effects
</commit_message>
<xml_diff>
--- a/docs/obbbafim/Effects of OBBBA and Tariffs on FIM.xlsx
+++ b/docs/obbbafim/Effects of OBBBA and Tariffs on FIM.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://brookingsinstitution-my.sharepoint.com/personal/sahmad_brookings_edu/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAhmad\Downloads\FIM\docs\obbbafim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="8_{A4F5FBC4-6C59-4563-A094-863C1F623D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F962A876-024F-45DA-A3C7-1684ACEA0178}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC69DEBA-A965-474F-BBED-522FC89D3008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72AE769E-C51D-4F87-9971-970B5B886A6C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{72AE769E-C51D-4F87-9971-970B5B886A6C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="NEW" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,17 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="17">
   <si>
     <t>Effects of OBBBA</t>
   </si>
   <si>
-    <t>Current FIM</t>
-  </si>
-  <si>
-    <t>Current FIM without OBBBA</t>
-  </si>
-  <si>
     <t>2025 Q2</t>
   </si>
   <si>
@@ -81,9 +74,6 @@
     <t>Current FIM without tariffs</t>
   </si>
   <si>
-    <t>new fim</t>
-  </si>
-  <si>
     <t>pre changes FIM</t>
   </si>
   <si>
@@ -91,6 +81,12 @@
   </si>
   <si>
     <t>post changes FIM without OBBBA</t>
+  </si>
+  <si>
+    <t>August</t>
+  </si>
+  <si>
+    <t>September</t>
   </si>
 </sst>
 </file>
@@ -138,10 +134,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -163,16 +162,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1133475</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:rowOff>34925</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>915599</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>525074</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -195,8 +194,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2838450" y="2362200"/>
-          <a:ext cx="4249349" cy="1695450"/>
+          <a:off x="0" y="2387600"/>
+          <a:ext cx="4252524" cy="1698625"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -525,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ECFED45-85A7-46EB-BA6E-79FB059E10A9}">
-  <dimension ref="A2:K12"/>
+  <dimension ref="A2:K25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="15.6328125" bestFit="1" customWidth="1"/>
@@ -539,24 +538,27 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -564,7 +566,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4">
         <v>-0.244775494829167</v>
@@ -577,7 +579,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H4">
         <v>-0.244775494829167</v>
@@ -592,7 +594,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5">
         <v>-3.1870410854322899E-2</v>
@@ -605,7 +607,7 @@
         <v>0.59987708355349312</v>
       </c>
       <c r="G5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H5">
         <v>-0.226791216752876</v>
@@ -620,7 +622,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6">
         <v>-0.36819629744312399</v>
@@ -637,7 +639,7 @@
         <v>0.21712408037607178</v>
       </c>
       <c r="G6" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H6">
         <v>-0.45121728224805602</v>
@@ -656,7 +658,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B7">
         <v>0.17754835712912601</v>
@@ -669,7 +671,7 @@
         <v>0.57480940076876397</v>
       </c>
       <c r="G7" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H7">
         <v>9.0269397362426701E-2</v>
@@ -684,7 +686,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B8">
         <v>-0.31455667513132601</v>
@@ -697,7 +699,7 @@
         <v>0.30164418888823696</v>
       </c>
       <c r="G8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H8">
         <v>-0.39836256599206799</v>
@@ -712,7 +714,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B9">
         <v>-0.45348329348996502</v>
@@ -725,7 +727,7 @@
         <v>0.251665075148712</v>
       </c>
       <c r="G9" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H9">
         <v>-0.54427302977775105</v>
@@ -740,7 +742,7 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B10">
         <v>-0.61858704819056198</v>
@@ -757,7 +759,7 @@
         <v>0.31335875068841024</v>
       </c>
       <c r="G10" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H10">
         <v>-0.70577816924638603</v>
@@ -776,7 +778,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B11">
         <v>-0.75821772384533004</v>
@@ -789,7 +791,7 @@
         <v>0.16099015753073498</v>
       </c>
       <c r="G11" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H11">
         <v>-0.83175475601170401</v>
@@ -804,7 +806,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B12">
         <v>-0.639050241881712</v>
@@ -817,7 +819,7 @@
         <v>0.15726850767336997</v>
       </c>
       <c r="G12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H12">
         <v>-0.71228889011569096</v>
@@ -829,328 +831,150 @@
         <f t="shared" si="1"/>
         <v>-0.22436350585965398</v>
       </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H15" t="s">
+        <v>10</v>
+      </c>
+      <c r="I15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H16" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16" t="s">
+        <v>11</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="7:11" x14ac:dyDescent="0.35">
+      <c r="G17" t="s">
+        <v>1</v>
+      </c>
+      <c r="H17" s="3">
+        <v>-0.62724129518848803</v>
+      </c>
+      <c r="I17" s="1">
+        <v>-0.3</v>
+      </c>
+      <c r="J17" s="1">
+        <f>H17-I17</f>
+        <v>-0.32724129518848805</v>
+      </c>
+    </row>
+    <row r="18" spans="7:11" x14ac:dyDescent="0.35">
+      <c r="G18" t="s">
+        <v>2</v>
+      </c>
+      <c r="H18" s="3">
+        <v>0.15065645415148901</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0.87</v>
+      </c>
+      <c r="J18" s="1">
+        <f t="shared" ref="J18:J25" si="2">H18-I18</f>
+        <v>-0.71934354584851101</v>
+      </c>
+    </row>
+    <row r="19" spans="7:11" x14ac:dyDescent="0.35">
+      <c r="G19" t="s">
+        <v>3</v>
+      </c>
+      <c r="H19" s="3">
+        <v>-0.129455533931744</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="J19" s="1">
+        <f t="shared" si="2"/>
+        <v>-0.79945553393174407</v>
+      </c>
+      <c r="K19" s="2">
+        <f>AVERAGE(J16:J19)</f>
+        <v>-0.46151009374218577</v>
+      </c>
+    </row>
+    <row r="20" spans="7:11" x14ac:dyDescent="0.35">
+      <c r="G20" t="s">
+        <v>4</v>
+      </c>
+      <c r="H20" s="3">
+        <v>0.412493312758139</v>
+      </c>
+      <c r="I20" s="1">
+        <v>0.93</v>
+      </c>
+      <c r="J20" s="1">
+        <f t="shared" si="2"/>
+        <v>-0.517506687241861</v>
+      </c>
+    </row>
+    <row r="21" spans="7:11" x14ac:dyDescent="0.35">
+      <c r="G21" t="s">
+        <v>5</v>
+      </c>
+      <c r="H21" s="3">
+        <v>-8.0426526834644504E-2</v>
+      </c>
+      <c r="I21" s="1">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="J21" s="1">
+        <f t="shared" si="2"/>
+        <v>-0.3704265268346445</v>
+      </c>
+    </row>
+    <row r="22" spans="7:11" x14ac:dyDescent="0.35">
+      <c r="G22" t="s">
+        <v>6</v>
+      </c>
+      <c r="H22" s="3">
+        <v>-0.23164761582804899</v>
+      </c>
+      <c r="I22" s="1">
+        <v>0.13</v>
+      </c>
+      <c r="J22" s="1">
+        <f t="shared" si="2"/>
+        <v>-0.361647615828049</v>
+      </c>
+    </row>
+    <row r="23" spans="7:11" x14ac:dyDescent="0.35">
+      <c r="G23" t="s">
+        <v>7</v>
+      </c>
+      <c r="H23" s="3">
+        <v>-0.42776992615857301</v>
+      </c>
+      <c r="I23" s="1">
+        <v>-0.06</v>
+      </c>
+      <c r="J23" s="1">
+        <f t="shared" si="2"/>
+        <v>-0.36776992615857301</v>
+      </c>
+      <c r="K23" s="2">
+        <f>AVERAGE(J20:J23)</f>
+        <v>-0.40433768901578188</v>
+      </c>
+    </row>
+    <row r="24" spans="7:11" x14ac:dyDescent="0.35">
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+    </row>
+    <row r="25" spans="7:11" x14ac:dyDescent="0.35">
+      <c r="J25" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{192B0D0E-CC33-414C-9F13-F76C8260EA91}">
-  <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.90625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="H2" t="s">
-        <v>1</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>3.1978474768033997E-2</v>
-      </c>
-      <c r="C3">
-        <v>-0.24</v>
-      </c>
-      <c r="D3" s="1">
-        <f>B3-C3</f>
-        <v>0.271978474768034</v>
-      </c>
-      <c r="G3" t="s">
-        <v>3</v>
-      </c>
-      <c r="H3">
-        <v>3.1978474768033997E-2</v>
-      </c>
-      <c r="I3">
-        <v>0.33197847476803399</v>
-      </c>
-      <c r="J3" s="1">
-        <f>H3-I3</f>
-        <v>-0.3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
-        <v>0.26493022087831197</v>
-      </c>
-      <c r="C4">
-        <v>-0.63</v>
-      </c>
-      <c r="D4" s="1">
-        <f t="shared" ref="D4:D11" si="0">B4-C4</f>
-        <v>0.89493022087831198</v>
-      </c>
-      <c r="G4" t="s">
-        <v>4</v>
-      </c>
-      <c r="H4">
-        <v>0.26493022087831197</v>
-      </c>
-      <c r="I4">
-        <v>0.525755130286928</v>
-      </c>
-      <c r="J4" s="1">
-        <f t="shared" ref="J4:J11" si="1">H4-I4</f>
-        <v>-0.26082490940861602</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>-0.20744973494473601</v>
-      </c>
-      <c r="C5">
-        <v>-0.65</v>
-      </c>
-      <c r="D5" s="1">
-        <f t="shared" si="0"/>
-        <v>0.44255026505526401</v>
-      </c>
-      <c r="E5" s="1">
-        <f>AVERAGE(D2:D5)</f>
-        <v>0.40236474017540247</v>
-      </c>
-      <c r="G5" t="s">
-        <v>5</v>
-      </c>
-      <c r="H5">
-        <v>-0.20744973494473601</v>
-      </c>
-      <c r="I5">
-        <v>0.249125039387324</v>
-      </c>
-      <c r="J5" s="1">
-        <f t="shared" si="1"/>
-        <v>-0.45657477433206001</v>
-      </c>
-      <c r="K5" s="1">
-        <f>AVERAGE(J2:J5)</f>
-        <v>-0.254349920935169</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>0.47607361294494899</v>
-      </c>
-      <c r="C6">
-        <v>-0.41</v>
-      </c>
-      <c r="D6" s="1">
-        <f t="shared" si="0"/>
-        <v>0.88607361294494891</v>
-      </c>
-      <c r="G6" t="s">
-        <v>6</v>
-      </c>
-      <c r="H6">
-        <v>0.47607361294494899</v>
-      </c>
-      <c r="I6">
-        <v>0.69634154085671796</v>
-      </c>
-      <c r="J6" s="1">
-        <f t="shared" si="1"/>
-        <v>-0.22026792791176897</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
-        <v>-0.115982217402605</v>
-      </c>
-      <c r="C7">
-        <v>-0.63</v>
-      </c>
-      <c r="D7" s="1">
-        <f t="shared" si="0"/>
-        <v>0.51401778259739506</v>
-      </c>
-      <c r="G7" t="s">
-        <v>7</v>
-      </c>
-      <c r="H7">
-        <v>-0.115982217402605</v>
-      </c>
-      <c r="I7">
-        <v>6.1105326298112397E-2</v>
-      </c>
-      <c r="J7" s="1">
-        <f t="shared" si="1"/>
-        <v>-0.17708754370071739</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>-0.25488464448468001</v>
-      </c>
-      <c r="C8">
-        <v>-0.71</v>
-      </c>
-      <c r="D8" s="1">
-        <f t="shared" si="0"/>
-        <v>0.45511535551531995</v>
-      </c>
-      <c r="G8" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8">
-        <v>-0.25488464448468001</v>
-      </c>
-      <c r="I8">
-        <v>-8.8692667153502699E-2</v>
-      </c>
-      <c r="J8" s="1">
-        <f t="shared" si="1"/>
-        <v>-0.1661919773311773</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>-0.41997834357757502</v>
-      </c>
-      <c r="C9">
-        <v>-0.75</v>
-      </c>
-      <c r="D9" s="1">
-        <f t="shared" si="0"/>
-        <v>0.33002165642242498</v>
-      </c>
-      <c r="E9" s="1">
-        <f>AVERAGE(D6:D9)</f>
-        <v>0.54630710187002229</v>
-      </c>
-      <c r="G9" t="s">
-        <v>9</v>
-      </c>
-      <c r="H9">
-        <v>-0.41997834357757502</v>
-      </c>
-      <c r="I9">
-        <v>-0.250167625586043</v>
-      </c>
-      <c r="J9" s="1">
-        <f t="shared" si="1"/>
-        <v>-0.16981071799153202</v>
-      </c>
-      <c r="K9" s="1">
-        <f>AVERAGE(J6:J9)</f>
-        <v>-0.18333954173379891</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>-0.65959177125745705</v>
-      </c>
-      <c r="C10">
-        <v>-0.92</v>
-      </c>
-      <c r="D10" s="1">
-        <f t="shared" si="0"/>
-        <v>0.26040822874254299</v>
-      </c>
-      <c r="G10" t="s">
-        <v>10</v>
-      </c>
-      <c r="H10">
-        <v>-0.65959177125745705</v>
-      </c>
-      <c r="I10">
-        <v>-0.47588569551266702</v>
-      </c>
-      <c r="J10" s="1">
-        <f t="shared" si="1"/>
-        <v>-0.18370607574479003</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11">
-        <v>-0.66913689549169197</v>
-      </c>
-      <c r="C11">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="D11" s="1">
-        <f t="shared" si="0"/>
-        <v>-0.80913689549169199</v>
-      </c>
-      <c r="G11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H11">
-        <v>-0.66913689549169197</v>
-      </c>
-      <c r="I11">
-        <v>-0.48792538425603699</v>
-      </c>
-      <c r="J11" s="1">
-        <f t="shared" si="1"/>
-        <v>-0.18121151123565499</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>